<commit_message>
realised xy histogram was being loaded flipped upside down verticallygit add . fixed that (changed definition of z linspace) and added title to interactive detector view plot
</commit_message>
<xml_diff>
--- a/wombat_Y2SiO5_example/Y2SiO5_reflections_angles.xlsx
+++ b/wombat_Y2SiO5_example/Y2SiO5_reflections_angles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>two theta (deg)</t>
+          <t>A4 (deg)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -459,6 +459,11 @@
           <t>z (m)</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>two theta (deg)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -481,6 +486,9 @@
       </c>
       <c r="G2" t="n">
         <v>-0.79931</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10.69134</v>
       </c>
     </row>
     <row r="3">
@@ -505,36 +513,42 @@
       <c r="G3" t="n">
         <v>-0</v>
       </c>
+      <c r="H3" t="n">
+        <v>48.90247</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="n">
-        <v>4</v>
-      </c>
       <c r="C4" t="n">
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>-4</v>
       </c>
       <c r="E4" t="n">
-        <v>-116.87136</v>
+        <v>15.68452</v>
       </c>
       <c r="F4" t="n">
-        <v>-72.072</v>
+        <v>-56.25807</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.00829</v>
+        <v>-0.031</v>
+      </c>
+      <c r="H4" t="n">
+        <v>56.25807</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -543,13 +557,16 @@
         <v>-4</v>
       </c>
       <c r="E5" t="n">
-        <v>15.68452</v>
+        <v>31.44333</v>
       </c>
       <c r="F5" t="n">
-        <v>-56.25807</v>
+        <v>-66.2405</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.031</v>
+        <v>-0.01784</v>
+      </c>
+      <c r="H5" t="n">
+        <v>66.2405</v>
       </c>
     </row>
     <row r="6">
@@ -557,19 +574,176 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-4</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-34.25322</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-66.91202</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.04416</v>
+      </c>
+      <c r="H6" t="n">
+        <v>66.91202</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="n">
         <v>4</v>
       </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-116.87136</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-72.072</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-0.00829</v>
+      </c>
+      <c r="H7" t="n">
+        <v>72.072</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-6</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.22973</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-94.33637</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-0.02658</v>
+      </c>
+      <c r="H8" t="n">
+        <v>94.33637</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-170.48089</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-110.08894</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.01784</v>
+      </c>
+      <c r="H9" t="n">
+        <v>110.08894</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-147.51378</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-111.75441</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>111.75441</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-80.80262999999999</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-113.31102</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-0.0408</v>
+      </c>
+      <c r="H11" t="n">
+        <v>113.31102</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>6</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
         <v>0.0045</v>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
preliminary wombatDMCpy how-to guide, and updated Y2SiO5 example
</commit_message>
<xml_diff>
--- a/wombat_Y2SiO5_example/Y2SiO5_reflections_angles.xlsx
+++ b/wombat_Y2SiO5_example/Y2SiO5_reflections_angles.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="J:\wombat_instrument_work\eulerian_cradle\Wombat_DMCpy\wombat_Y2SiO5_example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18546974-2A28-408D-A5BD-282B4D5AF71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A8FA2B-2345-4A05-BE93-D476D2AA9330}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6435" yWindow="1440" windowWidth="21600" windowHeight="12510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2415" yWindow="2160" windowWidth="21600" windowHeight="12510" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -406,12 +406,8 @@
   <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -451,16 +447,16 @@
         <v>0</v>
       </c>
       <c r="E2">
-        <v>-68.613759999999999</v>
+        <v>111.13418</v>
       </c>
       <c r="F2">
-        <v>-10.69134</v>
+        <v>-11.28567</v>
       </c>
       <c r="G2">
-        <v>-0.79930999999999996</v>
+        <v>-0.77851999999999999</v>
       </c>
       <c r="H2">
-        <v>10.69134</v>
+        <v>11.28567</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -477,16 +473,16 @@
         <v>2</v>
       </c>
       <c r="E3">
-        <v>-116.08781</v>
+        <v>63.783470000000001</v>
       </c>
       <c r="F3">
-        <v>-48.902470000000001</v>
+        <v>-48.88702</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>1.7729999999999999E-2</v>
       </c>
       <c r="H3">
-        <v>48.902470000000001</v>
+        <v>48.88702</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -503,16 +499,16 @@
         <v>-4</v>
       </c>
       <c r="E4">
-        <v>15.684519999999999</v>
+        <v>-164.50511</v>
       </c>
       <c r="F4">
-        <v>-56.258069999999996</v>
+        <v>-56.238849999999999</v>
       </c>
       <c r="G4">
-        <v>-3.1E-2</v>
+        <v>-3.5959999999999999E-2</v>
       </c>
       <c r="H4">
-        <v>56.258069999999996</v>
+        <v>56.238849999999999</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -529,16 +525,16 @@
         <v>-4</v>
       </c>
       <c r="E5">
-        <v>31.44333</v>
+        <v>-148.70690999999999</v>
       </c>
       <c r="F5">
-        <v>-66.240499999999997</v>
+        <v>-66.200940000000003</v>
       </c>
       <c r="G5">
-        <v>-1.7840000000000002E-2</v>
+        <v>-2.9649999999999999E-2</v>
       </c>
       <c r="H5">
-        <v>66.240499999999997</v>
+        <v>66.200940000000003</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -555,16 +551,16 @@
         <v>-4</v>
       </c>
       <c r="E6">
-        <v>-34.253219999999999</v>
+        <v>145.51604</v>
       </c>
       <c r="F6">
-        <v>-66.912019999999998</v>
+        <v>-66.971289999999996</v>
       </c>
       <c r="G6">
-        <v>-4.4159999999999998E-2</v>
+        <v>-3.3489999999999999E-2</v>
       </c>
       <c r="H6">
-        <v>66.912019999999998</v>
+        <v>66.971289999999996</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -581,16 +577,16 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>-116.87136</v>
+        <v>63.003720000000001</v>
       </c>
       <c r="F7">
-        <v>-72.072000000000003</v>
+        <v>-72.067570000000003</v>
       </c>
       <c r="G7">
-        <v>-8.2900000000000005E-3</v>
+        <v>1.1180000000000001E-2</v>
       </c>
       <c r="H7">
-        <v>72.072000000000003</v>
+        <v>72.067570000000003</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -607,16 +603,16 @@
         <v>-6</v>
       </c>
       <c r="E8">
-        <v>4.22973</v>
+        <v>-175.93306999999999</v>
       </c>
       <c r="F8">
-        <v>-94.336370000000002</v>
+        <v>-94.282589999999999</v>
       </c>
       <c r="G8">
-        <v>-2.6579999999999999E-2</v>
+        <v>-3.4169999999999999E-2</v>
       </c>
       <c r="H8">
-        <v>94.336370000000002</v>
+        <v>94.282589999999999</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -633,16 +629,16 @@
         <v>6</v>
       </c>
       <c r="E9">
-        <v>-170.48088999999999</v>
+        <v>9.3924400000000006</v>
       </c>
       <c r="F9">
-        <v>-110.08893999999999</v>
+        <v>-110.00223</v>
       </c>
       <c r="G9">
-        <v>1.7840000000000002E-2</v>
+        <v>2.9649999999999999E-2</v>
       </c>
       <c r="H9">
-        <v>110.08893999999999</v>
+        <v>110.00223</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -659,16 +655,16 @@
         <v>4</v>
       </c>
       <c r="E10">
-        <v>-147.51378</v>
+        <v>32.374839999999999</v>
       </c>
       <c r="F10">
-        <v>-111.75440999999999</v>
+        <v>-111.70426999999999</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>1.7729999999999999E-2</v>
       </c>
       <c r="H10">
-        <v>111.75440999999999</v>
+        <v>111.70426999999999</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -685,16 +681,16 @@
         <v>-4</v>
       </c>
       <c r="E11">
-        <v>-80.802629999999994</v>
+        <v>98.938720000000004</v>
       </c>
       <c r="F11">
-        <v>-113.31102</v>
+        <v>-113.49097</v>
       </c>
       <c r="G11">
-        <v>-4.0800000000000003E-2</v>
+        <v>-2.392E-2</v>
       </c>
       <c r="H11">
-        <v>113.31102</v>
+        <v>113.49097</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -711,7 +707,7 @@
         <v>6</v>
       </c>
       <c r="G12">
-        <v>4.4999999999999997E-3</v>
+        <v>2.103E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>